<commit_message>
Merge K sorted lists
</commit_message>
<xml_diff>
--- a/AmazonRecentInterviewQuestions/amazon_sde1_filtered_questions.xlsx
+++ b/AmazonRecentInterviewQuestions/amazon_sde1_filtered_questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NFRAC\Laboratory\Projects\Java\LeetCodeSolutions\AmazonRecentInterviewQuestions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9DE9D5-FE69-42EA-AAC9-D25A2C5E829F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713BA92A-C3C2-4059-B82E-3F2CBD2C2A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{57A929C8-930A-4808-BFA1-E940B7892482}"/>
   </bookViews>
@@ -2992,7 +2992,7 @@
       <c r="A82" t="s">
         <v>8</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>234</v>
       </c>
       <c r="C82" s="2" t="s">
@@ -3023,7 +3023,7 @@
       <c r="B84" t="s">
         <v>239</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C84" s="2" t="s">
         <v>240</v>
       </c>
       <c r="D84" t="s">
@@ -3062,7 +3062,7 @@
       <c r="A87" t="s">
         <v>8</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>248</v>
       </c>
       <c r="C87" s="2" t="s">
@@ -3090,7 +3090,7 @@
       <c r="A89" t="s">
         <v>8</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>254</v>
       </c>
       <c r="C89" s="2" t="s">
@@ -3104,7 +3104,7 @@
       <c r="A90" t="s">
         <v>8</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>257</v>
       </c>
       <c r="C90" s="2" t="s">
@@ -3497,8 +3497,9 @@
     <hyperlink ref="C109" r:id="rId88" xr:uid="{0C726199-E277-4D78-B4E4-2F9F38C7C18C}"/>
     <hyperlink ref="C110" r:id="rId89" xr:uid="{8C941205-88A6-4243-925C-7716F11B3B3F}"/>
     <hyperlink ref="C111" r:id="rId90" xr:uid="{83189FC4-0327-4B70-B9D7-DE95751C8E27}"/>
+    <hyperlink ref="C84" r:id="rId91" xr:uid="{F51CAEFD-286C-431E-8F9A-A4616D9F864D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId91"/>
+  <pageSetup orientation="portrait" r:id="rId92"/>
 </worksheet>
 </file>
</xml_diff>